<commit_message>
Khoa học 4, Đạo đức 4–5, LS&ĐL 4–5, Toán 4, Tiếng Việt 5: cột 7 bỏ dòng Năng lực số kiểu cũ không có trong giáo án (đồng bộ app bản 171)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/docs/lop4/Dao duc - Lop 4.xlsx
+++ b/assets/docs/lop4/Dao duc - Lop 4.xlsx
@@ -1032,11 +1032,7 @@
           <t>17</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>NLS-GT (Cơ bản 2): HS cùng xây dựng bản quy ước sử dụng phòng máy và bảng phân công trực nhật, mỗi tổ theo dõi và.</t>
-        </is>
-      </c>
+      <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1319,11 +1315,7 @@
           <t>26</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>NLS-GQVĐ (Cơ bản 2): Cho HS quan sát các cách tiêu tiền trên môi trường số: mua hàng qua mạng, nạp tiền vào trò chơi, mua.</t>
-        </is>
-      </c>
+      <c r="H29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">

</xml_diff>